<commit_message>
Updates following new data from Janelia
</commit_message>
<xml_diff>
--- a/gt_sources/eddison_et_al_2024/CX NP and NTs.xlsx
+++ b/gt_sources/eddison_et_al_2024/CX NP and NTs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/GD/LMBD/Papers/synister/drosophila_neuropeptides/gt_sources/eddison_et_al_2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A405CAA-CE04-6A43-A963-7B7EF7866641}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{851064AD-C4D1-3449-8F2F-F44805766952}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2420" yWindow="2640" windowWidth="33940" windowHeight="21580" xr2:uid="{8B69697B-4D45-A24E-B63F-052ECFDAAD09}"/>
+    <workbookView xWindow="3860" yWindow="1520" windowWidth="23440" windowHeight="19780" xr2:uid="{8B69697B-4D45-A24E-B63F-052ECFDAAD09}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2036,7 +2036,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2224,6 +2224,14 @@
       <color rgb="FF00B050"/>
       <name val="Calibri (Body)"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFFC000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -2324,7 +2332,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2433,6 +2441,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3484,7 +3495,7 @@
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A53" s="33" t="s">
+      <c r="A53" s="38" t="s">
         <v>22</v>
       </c>
       <c r="B53" s="24" t="s">
@@ -3512,7 +3523,7 @@
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A55" s="33" t="s">
+      <c r="A55" s="38" t="s">
         <v>24</v>
       </c>
       <c r="B55" s="20" t="s">
@@ -3526,7 +3537,7 @@
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A56" s="33" t="s">
+      <c r="A56" s="38" t="s">
         <v>25</v>
       </c>
       <c r="B56" s="20" t="s">
@@ -3595,7 +3606,7 @@
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A61" s="33" t="s">
+      <c r="A61" s="38" t="s">
         <v>29</v>
       </c>
       <c r="B61" s="20" t="s">
@@ -3620,7 +3631,7 @@
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A63" s="33" t="s">
+      <c r="A63" s="38" t="s">
         <v>31</v>
       </c>
       <c r="B63" s="27" t="s">
@@ -3634,7 +3645,7 @@
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A64" s="33" t="s">
+      <c r="A64" s="38" t="s">
         <v>32</v>
       </c>
       <c r="B64" s="24" t="s">
@@ -3651,7 +3662,7 @@
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A65" s="33" t="s">
+      <c r="A65" s="38" t="s">
         <v>33</v>
       </c>
       <c r="B65" s="20" t="s">
@@ -3690,7 +3701,7 @@
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A68" s="33" t="s">
+      <c r="A68" s="38" t="s">
         <v>36</v>
       </c>
       <c r="B68" s="20" t="s">
@@ -3704,7 +3715,7 @@
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A69" s="33" t="s">
+      <c r="A69" s="38" t="s">
         <v>110</v>
       </c>
       <c r="B69" s="24" t="s">
@@ -3718,7 +3729,7 @@
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A70" s="33" t="s">
+      <c r="A70" s="38" t="s">
         <v>37</v>
       </c>
       <c r="B70" s="20" t="s">
@@ -3914,7 +3925,7 @@
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A85" s="33" t="s">
+      <c r="A85" s="38" t="s">
         <v>112</v>
       </c>
       <c r="D85" s="3" t="s">

</xml_diff>